<commit_message>
allow for blank ORCID ID for contributor
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -1,37 +1,109 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://anu365-my.sharepoint.com/personal/u1173285_anu_edu_au/Documents/Documents/datacite/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59D2BFD380D5BB2CB42593563088B35299F0DF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3628B5AB-71CC-6E41-9469-AAFAC725CC0E}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="1620" yWindow="660" windowWidth="27780" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+  <si>
+    <t>Creator</t>
+  </si>
+  <si>
+    <t>Creator_ROR</t>
+  </si>
+  <si>
+    <t>Publisher</t>
+  </si>
+  <si>
+    <t>Contrib_ORCID</t>
+  </si>
+  <si>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Contrib_name</t>
+  </si>
+  <si>
+    <t>Pub_ROR</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>publication_year</t>
+  </si>
+  <si>
+    <t>doi</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>Phenomics Australia</t>
+  </si>
+  <si>
+    <t>https://ror.org/019wvm592</t>
+  </si>
+  <si>
+    <t>Lucy</t>
+  </si>
+  <si>
+    <t>Bradbury</t>
+  </si>
+  <si>
+    <t>Bradbury,Lucy</t>
+  </si>
+  <si>
+    <t>https://phenomicsaustralia.org.au/project</t>
+  </si>
+  <si>
+    <t>10.83986/nw5n-4375</t>
+  </si>
+  <si>
+    <t>Development of a Primary CNS Lymphoma (PCNSL)-Brain Organoid co-culture model</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +118,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,114 +442,84 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Creator</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Creator_ROR</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Publisher</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Contrib_ORCID</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Contrib_name</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Pub_ROR</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>publication_year</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>doi</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Phenomics Australia</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://ror.org/019wvm592</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Phenomics Australia</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://orcid.org/0000-0001-7475-4487</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Rossow, Nick</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://ror.org/019wvm592</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>https://phenomicsaustralia.org.au/project</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2">
         <v>2025</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>10.83986/9jmc-1k72</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>fresh123</t>
-        </is>
+      <c r="K2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
made more things optional arguments changed xlsx field names
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://anu365-my.sharepoint.com/personal/u1173285_anu_edu_au/Documents/Documents/datacite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59D2BFD380D5BB2CB42593563088B35299F0DF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3628B5AB-71CC-6E41-9469-AAFAC725CC0E}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_2B59D2BFD380D5BB2CB42593563088B35299F0DF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6957E0F1-3282-6942-8C85-27F9DA473F55}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="660" windowWidth="27780" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1640" yWindow="980" windowWidth="27780" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -446,7 +446,18 @@
   <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="34" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="65.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
modified DOI writeback to include full URL
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -1,109 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://anu365-my.sharepoint.com/personal/u1173285_anu_edu_au/Documents/Documents/datacite/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_2B59D2BFD380D5BB2CB42593563088B35299F0DF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6957E0F1-3282-6942-8C85-27F9DA473F55}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="1640" yWindow="980" windowWidth="27780" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
-  <si>
-    <t>Creator</t>
-  </si>
-  <si>
-    <t>Creator_ROR</t>
-  </si>
-  <si>
-    <t>Publisher</t>
-  </si>
-  <si>
-    <t>Contrib_ORCID</t>
-  </si>
-  <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Last Name</t>
-  </si>
-  <si>
-    <t>Contrib_name</t>
-  </si>
-  <si>
-    <t>Pub_ROR</t>
-  </si>
-  <si>
-    <t>url</t>
-  </si>
-  <si>
-    <t>publication_year</t>
-  </si>
-  <si>
-    <t>doi</t>
-  </si>
-  <si>
-    <t>title</t>
-  </si>
-  <si>
-    <t>Phenomics Australia</t>
-  </si>
-  <si>
-    <t>https://ror.org/019wvm592</t>
-  </si>
-  <si>
-    <t>Lucy</t>
-  </si>
-  <si>
-    <t>Bradbury</t>
-  </si>
-  <si>
-    <t>Bradbury,Lucy</t>
-  </si>
-  <si>
-    <t>https://phenomicsaustralia.org.au/project</t>
-  </si>
-  <si>
-    <t>10.83986/nw5n-4375</t>
-  </si>
-  <si>
-    <t>Development of a Primary CNS Lymphoma (PCNSL)-Brain Organoid co-culture model</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -118,43 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -442,95 +420,130 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="34" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="65.83203125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>creator</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>creator_ror</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>publisher</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>contrib_orcid</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>first name</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>last name</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>contrib_name</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>pub_ror</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>publication_year</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>doi</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>project title</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2">
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Phenomics Australia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://ror.org/019wvm592</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Phenomics Australia</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Lucy</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Bradbury</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Bradbury,Lucy</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://ror.org/019wvm592</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://phenomicsaustralia.org.au/project</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
         <v>2025</v>
       </c>
-      <c r="K2" t="s">
-        <v>18</v>
-      </c>
-      <c r="L2" t="s">
-        <v>19</v>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.83986/vf32-2x34</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Development of a Primary CNS Lymphoma (PCNSL)-Brain Organoid co-culture model</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
script now looks for a sheet called "sheet1" added producer ror to new contributor
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -1,37 +1,109 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://anu365-my.sharepoint.com/personal/u1173285_anu_edu_au/Documents/Documents/datacite/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_2B59D2BFD3F0DCB2E716CA50593088B35299F037" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD25FCA3-9111-4544-9D77-3A0493786949}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="1100" yWindow="1800" windowWidth="28300" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+  <si>
+    <t>creator</t>
+  </si>
+  <si>
+    <t>creator_ror</t>
+  </si>
+  <si>
+    <t>publisher</t>
+  </si>
+  <si>
+    <t>contrib_orcid</t>
+  </si>
+  <si>
+    <t>first name</t>
+  </si>
+  <si>
+    <t>last name</t>
+  </si>
+  <si>
+    <t>contrib_name</t>
+  </si>
+  <si>
+    <t>pub_ror</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>publication_year</t>
+  </si>
+  <si>
+    <t>doi</t>
+  </si>
+  <si>
+    <t>project title</t>
+  </si>
+  <si>
+    <t>Phenomics Australia</t>
+  </si>
+  <si>
+    <t>https://ror.org/019wvm592</t>
+  </si>
+  <si>
+    <t>Lucy</t>
+  </si>
+  <si>
+    <t>Bradbury</t>
+  </si>
+  <si>
+    <t>Bradbury,Lucy</t>
+  </si>
+  <si>
+    <t>https://phenomicsaustralia.org.au/project</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.83986/vf32-2x34</t>
+  </si>
+  <si>
+    <t>Development of a Primary CNS Lymphoma (PCNSL)-Brain Organoid co-culture model</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +118,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,130 +442,94 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="34" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="65.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>creator</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>creator_ror</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>publisher</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>contrib_orcid</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>first name</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>last name</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>contrib_name</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>pub_ror</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>publication_year</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>doi</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>project title</t>
-        </is>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Phenomics Australia</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://ror.org/019wvm592</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Phenomics Australia</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Lucy</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Bradbury</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Bradbury,Lucy</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>https://ror.org/019wvm592</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://phenomicsaustralia.org.au/project</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2">
         <v>2025</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.83986/vf32-2x34</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Development of a Primary CNS Lymphoma (PCNSL)-Brain Organoid co-culture model</t>
-        </is>
+      <c r="K2" t="s">
+        <v>18</v>
+      </c>
+      <c r="L2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>